<commit_message>
Refresh flagship weekly analysis from revised 7.27-8.2 report
Co-authored-by: ghg131419-cloud <ghg131419-cloud@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/天猫近3月数据_分析结果/旗舰店周报_利润下降原因分析.xlsx
+++ b/天猫近3月数据_分析结果/旗舰店周报_利润下降原因分析.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="01-利润下降原因" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="02-关键周对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="03-口径说明" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="02-相对上一版变化" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="03-关键周对比" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,10 +69,6 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -134,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,14 +177,10 @@
     <xf numFmtId="10" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -278,7 +270,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>推广后利润周趋势</a:t>
+              <a:t>推广后利润周趋势（修订后）</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -688,21 +680,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>从《天猫旗舰店周报》看利润下降原因</t>
+          <t>从《天猫旗舰店周报》（已修改）看利润下降原因</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据来源：天猫旗舰店周报_7.27-8.2.csv｜店铺级｜拆解：推广后变化 ≈ 推广前变化 − 推广投入变化</t>
+          <t>数据来源：天猫旗舰店周报_7.27-8.2.csv（用户修订版）｜店铺级｜推广后变化 ≈ 推广前变化 − 推广投入变化</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>一、利润下降原因结论</t>
+          <t>一、利润下降原因（按修订后数据）</t>
         </is>
       </c>
     </row>
@@ -718,73 +710,73 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="46" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>总览：近3个月店铺推广后利润多数为负。7月相对较好周是 7.6-7.12（-4109），随后走弱：7.13 -5144 → 7.20 -5582；7.27 回升到 -5089，8.3 又落到 -5821。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
+          <t>修订说明：相对上一版变化：6.1-6.7（推广后利润:3605.0-&gt;-7458.0）；6.15-6.21（推广后利润:3605.0-&gt;-7953.0）；6.22-6.28（推广后利润:3605.0-&gt;-7765.0）；6.8-6.14（推广后利润:3605.0-&gt;-8672.0）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>第一波下降（7.6→7.13）：推广后 -4109→-5144（-1035）。推广前利润 -3160，推广投入 -2604。主因：推广前利润下降（GMV同步下滑），不是推广费上升（推广费其实在降）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
+          <t>总览：7月较好周 7.6-7.12（推广后 -4109）后走弱；7.13 -5144 → 7.20 -5582；7.27 回升至 -5089；8.3 再降至 -5821。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="5" t="n">
         <v>3</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>第二波下降（7.13→7.20）：推广后 -5144→-5582（-438）。推广前 -156，推广投入 +607。主因：推广费上升，叠加推广前利润继续小幅走弱。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+          <t>第一波（7.6→7.13）：推广后 -4109→-5144（-1035）。推广前 -3160，推广投入 -2604 → 主要是推广前利润下降。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>7.27当周（相对7.20）：推广后改善到 -5089（+493）。推广前回升 +1491 大于推广投入增加 +1028，故利润好转。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
+          <t>第二波（7.13→7.20）：推广后 -5144→-5582（-438）。推广前 -156，推广投入 +607 → 主要是推广费上升。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
       <c r="A10" s="5" t="n">
         <v>5</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>第三波下降（7.27→8.3）：推广后 -5089→-5821（-732）。推广前虽升 +2413，但推广投入大增 +3049，推广费上升吃掉了增量利润。主因：推广费上升。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
+          <t>7.27当周（相对7.20）：推广后 -5582→-5089（+493）。推广前回升超过推广费增加，利润改善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>结论（针对这份周报）：近期利润下降不是单一原因——7月中上旬主要是“生意/推广前利润走弱”；7月下旬至8月初更多是“推广费抬升过快”。店铺级报告无法定位到具体商品ID。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
+          <t>第三波（7.27→8.3）：推广后 -5089→-5821（-732）。推广前 +2413，推广投入 +3049 → 主要是推广费上升。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
       <c r="A12" s="5" t="n">
         <v>7</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>数据提示：6.1-6.7 至 6.22-6.28 四周推广后利润均为 3605，疑似填报重复/口径异常，分析时不作为可靠基线。</t>
+          <t>一句话：近期利润变差 = 先是推广前利润/生意走弱，后是推广费抬升过快。店铺周报无法定位商品ID。6月推广后利润已区分：[-7458.0, -8672.0, -7953.0, -7765.0]</t>
         </is>
       </c>
     </row>
@@ -826,11 +818,6 @@
           <t>主因判断</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -857,11 +844,6 @@
           <t>主要是推广前利润下降</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>GMV下滑，推广费同步下降，但前利润掉更多</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -888,11 +870,6 @@
           <t>主要是推广费上升</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>前利润略降，推广费明显抬升</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -919,11 +896,6 @@
           <t>本期改善</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>前利润回升超过推广费增加</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -948,11 +920,6 @@
       <c r="F20" s="8" t="inlineStr">
         <is>
           <t>主要是推广费上升</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>前利润升，但推广投入升幅更大</t>
         </is>
       </c>
     </row>
@@ -1114,74 +1081,74 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>6.1-6.7</t>
         </is>
       </c>
-      <c r="B28" s="14" t="n">
+      <c r="B28" s="10" t="n">
         <v>123012</v>
       </c>
-      <c r="C28" s="14" t="n">
+      <c r="C28" s="10" t="n">
         <v>14905</v>
       </c>
-      <c r="D28" s="15" t="n">
+      <c r="D28" s="9" t="n">
         <v>-1629</v>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="10" t="n">
         <v>20101</v>
       </c>
-      <c r="F28" s="15" t="n">
+      <c r="F28" s="9" t="n">
         <v>-2766</v>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>3605</v>
-      </c>
-      <c r="H28" s="14" t="n">
-        <v>10447</v>
-      </c>
-      <c r="I28" s="16" t="n">
+      <c r="G28" s="9" t="n">
+        <v>-7458</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>-616</v>
+      </c>
+      <c r="I28" s="17" t="n">
         <v>0.1816</v>
       </c>
-      <c r="J28" s="13" t="inlineStr">
-        <is>
-          <t>改善/持平</t>
+      <c r="J28" s="8" t="inlineStr">
+        <is>
+          <t>主要是推广前利润下降</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>6.8-6.14</t>
         </is>
       </c>
-      <c r="B29" s="14" t="n">
+      <c r="B29" s="10" t="n">
         <v>113858</v>
       </c>
-      <c r="C29" s="14" t="n">
+      <c r="C29" s="10" t="n">
         <v>13782</v>
       </c>
-      <c r="D29" s="15" t="n">
+      <c r="D29" s="9" t="n">
         <v>-1123</v>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="E29" s="10" t="n">
         <v>20196</v>
       </c>
-      <c r="F29" s="14" t="n">
+      <c r="F29" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>3605</v>
-      </c>
-      <c r="H29" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="16" t="n">
+      <c r="G29" s="9" t="n">
+        <v>-8672</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>-1214</v>
+      </c>
+      <c r="I29" s="17" t="n">
         <v>0.197</v>
       </c>
-      <c r="J29" s="13" t="inlineStr">
-        <is>
-          <t>改善/持平</t>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>主要是推广前利润下降</t>
         </is>
       </c>
     </row>
@@ -1206,11 +1173,11 @@
       <c r="F30" s="15" t="n">
         <v>-706</v>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>3605</v>
-      </c>
-      <c r="H30" s="18" t="n">
-        <v>0</v>
+      <c r="G30" s="15" t="n">
+        <v>-7953</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>719</v>
       </c>
       <c r="I30" s="16" t="n">
         <v>0.1905</v>
@@ -1242,11 +1209,11 @@
       <c r="F31" s="15" t="n">
         <v>-2439</v>
       </c>
-      <c r="G31" s="14" t="n">
-        <v>3605</v>
-      </c>
-      <c r="H31" s="18" t="n">
-        <v>0</v>
+      <c r="G31" s="15" t="n">
+        <v>-7765</v>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>188</v>
       </c>
       <c r="I31" s="16" t="n">
         <v>0.1956</v>
@@ -1258,38 +1225,38 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>6.29-7.5</t>
         </is>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="14" t="n">
         <v>100176</v>
       </c>
-      <c r="C32" s="10" t="n">
+      <c r="C32" s="14" t="n">
         <v>12985</v>
       </c>
-      <c r="D32" s="10" t="n">
+      <c r="D32" s="14" t="n">
         <v>1263</v>
       </c>
-      <c r="E32" s="10" t="n">
+      <c r="E32" s="14" t="n">
         <v>17357</v>
       </c>
-      <c r="F32" s="10" t="n">
+      <c r="F32" s="14" t="n">
         <v>306</v>
       </c>
-      <c r="G32" s="9" t="n">
+      <c r="G32" s="15" t="n">
         <v>-5230</v>
       </c>
-      <c r="H32" s="9" t="n">
-        <v>-8835</v>
-      </c>
-      <c r="I32" s="17" t="n">
+      <c r="H32" s="14" t="n">
+        <v>2535</v>
+      </c>
+      <c r="I32" s="16" t="n">
         <v>0.1888</v>
       </c>
-      <c r="J32" s="8" t="inlineStr">
-        <is>
-          <t>主要是推广费上升</t>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>改善/持平</t>
         </is>
       </c>
     </row>
@@ -1489,222 +1456,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
-        <is>
-          <t>关键周绝对数对比</t>
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>修订版 vs 上一版差异明细</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>指标</t>
+          <t>周次</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>7.6-7.12</t>
+          <t>字段</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>7.13-7.19</t>
+          <t>旧值</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>7.20-7.26</t>
+          <t>新值</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>7.27-8.2</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>8.3-8.9</t>
+          <t>差额</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>GMV</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="n">
-        <v>131865</v>
+          <t>6.1-6.7</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>推广后利润</t>
+        </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>109087</v>
-      </c>
-      <c r="D4" s="14" t="n">
-        <v>107560</v>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>118941</v>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>135684</v>
+        <v>3605</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>-7458</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>-11063</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>去退金额</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n">
-        <v>120260</v>
+          <t>6.15-6.21</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>推广后利润</t>
+        </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>100078</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <v>98481</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>107318</v>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>121296</v>
+        <v>3605</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>-7953</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>-11558</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>推广前利润</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
-        <v>16861</v>
+          <t>6.22-6.28</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>推广后利润</t>
+        </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>13701</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>13545</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>15036</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>17449</v>
+        <v>3605</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>-7765</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>-11370</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>推广投入</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="n">
-        <v>20174</v>
+          <t>6.8-6.14</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>推广后利润</t>
+        </is>
       </c>
       <c r="C7" s="14" t="n">
-        <v>17570</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>18177</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>19205</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>22254</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>推广产出</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>96278</v>
-      </c>
-      <c r="C8" s="14" t="n">
-        <v>80093</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>85856</v>
-      </c>
-      <c r="E8" s="14" t="n">
-        <v>92707</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>98839</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>其他费用</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n">
-        <v>2054</v>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>2405</v>
-      </c>
-      <c r="D9" s="14" t="n">
-        <v>2097</v>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>2127</v>
-      </c>
-      <c r="F9" s="14" t="n">
-        <v>2412</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>推广后利润</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="n">
-        <v>-4109</v>
-      </c>
-      <c r="C10" s="15" t="n">
-        <v>-5144</v>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>-5582</v>
-      </c>
-      <c r="E10" s="15" t="n">
-        <v>-5089</v>
-      </c>
-      <c r="F10" s="15" t="n">
-        <v>-5821</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>推广费率</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>0.1678</v>
-      </c>
-      <c r="C11" s="20" t="n">
-        <v>0.1756</v>
-      </c>
-      <c r="D11" s="20" t="n">
-        <v>0.1846</v>
-      </c>
-      <c r="E11" s="20" t="n">
-        <v>0.179</v>
-      </c>
-      <c r="F11" s="20" t="n">
-        <v>0.1835</v>
+        <v>3605</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>-8672</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>-12277</v>
       </c>
     </row>
   </sheetData>
@@ -1718,45 +1588,200 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
-        <is>
-          <t>口径说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
-        <is>
-          <t>本报告仅基于《天猫旗舰店周报》店铺合计数据，不能定位到具体商品ID。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
-        <is>
-          <t>下降主因规则：当周推广后利润环比为负时，比较“推广前利润减少”与“推广投入增加”谁贡献更大。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
-        <is>
-          <t>6.1-6.7 至 6.22-6.28 四周推广后利润同为3605，疑似异常，不作为基线。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>若需ID级归因，请提供对应周的《天猫ID周损益》文件。</t>
-        </is>
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>关键周绝对数（修订后）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>7.6-7.12</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>7.13-7.19</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>7.20-7.26</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>7.27-8.2</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>8.3-8.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>131865</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>109087</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>107560</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>118941</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>135684</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>去退金额</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>120260</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>100078</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>98481</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>107318</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>121296</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>推广前利润</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>16861</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>13701</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>13545</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>15036</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>17449</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>推广投入</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>20174</v>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>17570</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>18177</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>19205</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>22254</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>其他费用</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>2054</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>2405</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>2097</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>2127</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>2412</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>推广后利润</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>-4109</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>-5144</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>-5582</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>-5089</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>-5821</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>推广费率</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>0.1678</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>0.1756</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>0.1846</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>0.1835</v>
       </c>
     </row>
   </sheetData>

</xml_diff>